<commit_message>
add first floor expo areas
also changed js to be less specific about expo area labeling and styling; easier to change in the emptyspace excel and re-run the r script
</commit_message>
<xml_diff>
--- a/data/emptyspace.xlsx
+++ b/data/emptyspace.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/chloeedwards_tudelft_nl/Documents/Documents/GitHub/Digital-Twin-3/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{21B08916-1BD2-4732-92A8-8421AD5A9288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFA90493-85EA-47F0-8D09-07F50A027CFF}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="8_{21B08916-1BD2-4732-92A8-8421AD5A9288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6B851D7-9864-4068-A703-4A665EF5CE59}"/>
   <bookViews>
-    <workbookView xWindow="15375" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{4B1CBE11-476F-424F-AA1E-E50E55F321CD}"/>
+    <workbookView xWindow="22275" yWindow="-12585" windowWidth="21600" windowHeight="11175" xr2:uid="{4B1CBE11-476F-424F-AA1E-E50E55F321CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
   <si>
     <t>Name</t>
   </si>
@@ -99,6 +99,18 @@
   </si>
   <si>
     <t>AS</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Art Library</t>
+  </si>
+  <si>
+    <t>Heritage Vitrine</t>
+  </si>
+  <si>
+    <t>Expo</t>
   </si>
 </sst>
 </file>
@@ -470,11 +482,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{547D9816-D7CE-41CE-999D-C20DD7CBA263}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.08984375" customWidth="1"/>
+    <col min="3" max="3" width="13.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -603,6 +616,48 @@
         <v>19</v>
       </c>
     </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>130</v>
+      </c>
+      <c r="B10">
+        <v>132</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>152</v>
+      </c>
+      <c r="B11">
+        <v>154</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>178</v>
+      </c>
+      <c r="B12">
+        <v>180</v>
+      </c>
+      <c r="C12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>